<commit_message>
Update industry analysis report to include missing features
Add a sheet detailing missing features for each industry to the SwachERP industry fit analysis Excel report.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: e70c97c4-e099-455a-b9ae-aa9a0dedb718
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 11bf38b8-ce6c-4a31-9df6-e55f226394fe
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/713657ac-53c6-43a9-97a8-ef2697ef92d9/e70c97c4-e099-455a-b9ae-aa9a0dedb718/x05r5IY
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/SwachERP_Industry_Fit_Analysis.xlsx
+++ b/SwachERP_Industry_Fit_Analysis.xlsx
@@ -3,11 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="All Industries" sheetId="1" r:id="rId1"/>
-    <sheet name="Excellent Fit" sheetId="2" r:id="rId2"/>
-    <sheet name="Good Fit" sheetId="3" r:id="rId3"/>
-    <sheet name="Partial Fit" sheetId="4" r:id="rId4"/>
-    <sheet name="Poor Fit" sheetId="5" r:id="rId5"/>
+    <sheet name="Industry Fit Summary" sheetId="1" r:id="rId1"/>
+    <sheet name="Gaps &amp; What's Missing" sheetId="2" r:id="rId2"/>
+    <sheet name="New Modules to Build" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -419,15 +417,21 @@
       <c r="C1" t="str">
         <v/>
       </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Generated on: 7/5/2026</v>
+        <v>Generated: 07 May 2026</v>
       </c>
       <c r="B2" t="str">
         <v/>
       </c>
       <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
         <v/>
       </c>
     </row>
@@ -724,32 +728,64 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:E23"/>
   <cols>
-    <col min="1" max="1" width="42.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="80.83203125" customWidth="1"/>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="70.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>SwachERP — Industry Fit Analysis</v>
+        <v>SwachERP — Gaps &amp; Missing Features</v>
+      </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v/>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v/>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Tier: Excellent Fit (85–100%)</v>
+        <v>Generated: 07 May 2026</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Industry / Segment</v>
+        <v>INDUSTRY</v>
       </c>
       <c r="B4" t="str">
-        <v>Fit %</v>
+        <v>CURRENT FIT %</v>
       </c>
       <c r="C4" t="str">
-        <v>Details</v>
+        <v>WHAT'S MISSING</v>
+      </c>
+      <c r="D4" t="str">
+        <v>PRIORITY</v>
+      </c>
+      <c r="E4" t="str">
+        <v>EFFORT TO BUILD</v>
       </c>
     </row>
     <row r="5">
@@ -760,7 +796,13 @@
         <v>95%</v>
       </c>
       <c r="C5" t="str">
-        <v>Production/BOM, Quality, Inventory, Gatepasses, Maintenance, Purchase, Accounting</v>
+        <v>IoT machine integration, shop-floor app</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Low</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Medium</v>
       </c>
     </row>
     <row r="6">
@@ -771,7 +813,13 @@
         <v>93%</v>
       </c>
       <c r="C6" t="str">
-        <v>Invoicing, Multi-warehouse, Purchase, Sales Orders, CRM, GRN, GST</v>
+        <v>B2B customer portal, online order placement</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Medium</v>
       </c>
     </row>
     <row r="7">
@@ -782,7 +830,13 @@
         <v>91%</v>
       </c>
       <c r="C7" t="str">
-        <v>Dedicated POS module, Inventory, Invoicing, GST</v>
+        <v>Loyalty programme, gift card management</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Small</v>
       </c>
     </row>
     <row r="8">
@@ -793,7 +847,13 @@
         <v>90%</v>
       </c>
       <c r="C8" t="str">
-        <v>Full 12-tab Education ERP — students, fees, attendance, timetable, library, transport</v>
+        <v>Online exam / LMS, parent mobile app</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Large</v>
       </c>
     </row>
     <row r="9">
@@ -804,293 +864,469 @@
         <v>88%</v>
       </c>
       <c r="C9" t="str">
-        <v>Projects, Timesheets, Expense Claims, CRM, Invoicing, HR &amp; Payroll</v>
+        <v>Bug/ticket tracker, sprint boards</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Low</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Medium</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Professional Services (CA, Law, Consulting)</v>
+        <v>Professional Services</v>
       </c>
       <c r="B10" t="str">
         <v>86%</v>
       </c>
       <c r="C10" t="str">
-        <v>Projects, Timesheets, Invoicing, TDS, Accounting, CRM</v>
+        <v>Document e-signing, client portal</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Healthcare / Clinics</v>
+      </c>
+      <c r="B11" t="str">
+        <v>82%</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Pharmacy dispensing, LIMS, OT scheduling</v>
+      </c>
+      <c r="D11" t="str">
+        <v>High</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Large</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Logistics / Transport</v>
+      </c>
+      <c r="B12" t="str">
+        <v>82%</v>
+      </c>
+      <c r="C12" t="str">
+        <v>GPS/live tracking, ePOD, driver app</v>
+      </c>
+      <c r="D12" t="str">
+        <v>High</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Large</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Real Estate / Construction</v>
+      </c>
+      <c r="B13" t="str">
+        <v>80%</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Site attendance, contractor billing, RERA reports</v>
+      </c>
+      <c r="D13" t="str">
+        <v>High</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Agriculture / Agri-business</v>
+      </c>
+      <c r="B14" t="str">
+        <v>78%</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Crop insurance, mandi price integration, FPO module</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>NGO / Non-profit</v>
+      </c>
+      <c r="B15" t="str">
+        <v>72%</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Donor management, grant tracking, 80G receipts</v>
+      </c>
+      <c r="D15" t="str">
+        <v>High</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Pharma Distribution</v>
+      </c>
+      <c r="B16" t="str">
+        <v>70%</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Expiry alerts, Schedule-H drug tracking, FIFO batch</v>
+      </c>
+      <c r="D16" t="str">
+        <v>High</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Restaurant / Food Service</v>
+      </c>
+      <c r="B17" t="str">
+        <v>45%</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Table management, KOT printing, recipe costing, Swiggy/Zomato sync</v>
+      </c>
+      <c r="D17" t="str">
+        <v>High</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Large</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Hotel / Hospitality</v>
+      </c>
+      <c r="B18" t="str">
+        <v>35%</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Room booking, housekeeping, reservation system, OTA sync</v>
+      </c>
+      <c r="D18" t="str">
+        <v>High</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Large</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>E-commerce</v>
+      </c>
+      <c r="B19" t="str">
+        <v>50%</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Shopify/WooCommerce sync, returns portal, courier integration</v>
+      </c>
+      <c r="D19" t="str">
+        <v>High</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Large</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Jewellery / Gold</v>
+      </c>
+      <c r="B20" t="str">
+        <v>20%</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Gold rate management, ornament stock by weight/purity, karigar job work, hallmarking, gold loans</v>
+      </c>
+      <c r="D20" t="str">
+        <v>High</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Large</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>NBFC / Microfinance / Nidhi</v>
+      </c>
+      <c r="B21" t="str">
+        <v>25%</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Loan origination, EMI scheduler, KYC, member accounts, FD/RD deposits, RBI compliance</v>
+      </c>
+      <c r="D21" t="str">
+        <v>High</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Large</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Insurance</v>
+      </c>
+      <c r="B22" t="str">
+        <v>20%</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Policy management, claims, agent commissions, renewal reminders</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Large</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Hospital (large)</v>
+      </c>
+      <c r="B23" t="str">
+        <v>40%</v>
+      </c>
+      <c r="C23" t="str">
+        <v>OT scheduling, LIMS, pharmacy dispensing, doctor scheduling, insurance billing</v>
+      </c>
+      <c r="D23" t="str">
+        <v>High</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Large</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E23"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:E12"/>
   <cols>
-    <col min="1" max="1" width="42.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="80.83203125" customWidth="1"/>
+    <col min="1" max="1" width="26.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="72.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>SwachERP — Industry Fit Analysis</v>
+        <v>SwachERP — Recommended New Modules to Build</v>
+      </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v/>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v/>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Tier: Good Fit (65–84%)</v>
+        <v>These additions would increase overall industry coverage significantly</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Industry / Segment</v>
+        <v>MODULE TO BUILD</v>
       </c>
       <c r="B4" t="str">
-        <v>Fit %</v>
+        <v>TARGET INDUSTRY</v>
       </c>
       <c r="C4" t="str">
-        <v>Details</v>
+        <v>MARKET SIZE (INDIA)</v>
+      </c>
+      <c r="D4" t="str">
+        <v>KEY FEATURES NEEDED</v>
+      </c>
+      <c r="E4" t="str">
+        <v>ESTIMATED EFFORT</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Healthcare / Clinics</v>
+        <v>Gold / Jewellery ERP</v>
       </c>
       <c r="B5" t="str">
-        <v>82%</v>
+        <v>Jewellers, Gold loan shops</v>
       </c>
       <c r="C5" t="str">
-        <v>Dedicated Healthcare module (OPD/IPD/Wards), HR, Accounting — missing pharmacy inventory</v>
+        <v>4+ lakh jewellery shops</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Gold rate mgmt, ornament stock by weight/purity/making charges, karigar job work, hallmarking, gold loans</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Large</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Logistics / Transport</v>
+        <v>NBFC / Nidhi / MFI ERP</v>
       </c>
       <c r="B6" t="str">
-        <v>82%</v>
+        <v>Cooperatives, Nidhi companies</v>
       </c>
       <c r="C6" t="str">
-        <v>Dedicated Logistics module, Fleet, Consignment Notes — missing GPS/live tracking</v>
+        <v>13,000+ Nidhi companies</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Loan origination, EMI scheduler, KYC, member accounts, FD/RD deposits, RBI reports</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Large</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Real Estate / Construction</v>
+        <v>Restaurant / F&amp;B ERP</v>
       </c>
       <c r="B7" t="str">
-        <v>80%</v>
+        <v>Restaurants, cloud kitchens</v>
       </c>
       <c r="C7" t="str">
-        <v>Dedicated RE module + Project Management, BOQ, Milestones — missing site attendance</v>
+        <v>7.5 million+ outlets</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Table management, KOT, recipe costing, Swiggy/Zomato sync, chef orders</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Medium</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Agriculture / Agri-business</v>
+        <v>Hotel / Hospitality ERP</v>
       </c>
       <c r="B8" t="str">
-        <v>78%</v>
+        <v>Hotels, resorts, guesthouses</v>
       </c>
       <c r="C8" t="str">
-        <v>Dedicated Agriculture module, Procurement, Commodity Prices — missing crop insurance</v>
+        <v>1.5 lakh+ hotels</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Room booking, housekeeping, reservation, OTA sync, banquet mgmt</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Large</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>NGO / Non-profit</v>
+        <v>Pharmacy ERP</v>
       </c>
       <c r="B9" t="str">
-        <v>72%</v>
+        <v>Medical stores, hospital pharma</v>
       </c>
       <c r="C9" t="str">
-        <v>Accounting, HR, Projects, Expense Claims — missing donor management</v>
+        <v>9 lakh+ pharmacies</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Drug scheduling, expiry tracking, FIFO, Schedule-H, doctor-wise sales</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Medium</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Pharma Distribution</v>
+        <v>Hospital (Advanced)</v>
       </c>
       <c r="B10" t="str">
-        <v>70%</v>
+        <v>Multi-specialty hospitals</v>
       </c>
       <c r="C10" t="str">
-        <v>Inventory, Batch/Lot tracking, Purchase, GST — missing expiry-based stock alerts</v>
+        <v>65,000+ hospitals</v>
+      </c>
+      <c r="D10" t="str">
+        <v>OT scheduling, LIMS, ward management, insurance billing, doctor roster</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Large</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>E-commerce ERP</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Online sellers, D2C brands</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Growing rapidly</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Shopify/WooCommerce sync, returns portal, courier integration, marketplace orders</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>NGO / Trust ERP</v>
+      </c>
+      <c r="B12" t="str">
+        <v>NGOs, charities, trusts</v>
+      </c>
+      <c r="C12" t="str">
+        <v>3+ lakh NGOs</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Donor management, grant tracking, 80G receipts, CSR reporting</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Small</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C10"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
-  <cols>
-    <col min="1" max="1" width="42.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="80.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>SwachERP — Industry Fit Analysis</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Tier: Partial Fit (40–64%)</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Industry / Segment</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Fit %</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Details</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Restaurant / Food Service</v>
-      </c>
-      <c r="B5" t="str">
-        <v>45%</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Basic POS works — missing table management, KOT, recipe costing</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Hotel / Hospitality</v>
-      </c>
-      <c r="B6" t="str">
-        <v>35%</v>
-      </c>
-      <c r="C6" t="str">
-        <v>No room booking, housekeeping, or reservation system</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>E-commerce</v>
-      </c>
-      <c r="B7" t="str">
-        <v>50%</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Inventory + Invoicing work — no Shopify/WooCommerce sync, no returns portal</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Jewellery / Gold</v>
-      </c>
-      <c r="B8" t="str">
-        <v>20%</v>
-      </c>
-      <c r="C8" t="str">
-        <v>No gold rate management, karigar job work, hallmarking, or gold loan module</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-  </mergeCells>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
-  <cols>
-    <col min="1" max="1" width="42.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="80.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>SwachERP — Industry Fit Analysis</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Tier: Poor Fit (Under 40%)</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Industry / Segment</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Fit %</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Details</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>NBFC / Microfinance / Nidhi</v>
-      </c>
-      <c r="B5" t="str">
-        <v>25%</v>
-      </c>
-      <c r="C5" t="str">
-        <v>No loan origination, EMI scheduler, KYC, RBI compliance reports</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Insurance</v>
-      </c>
-      <c r="B6" t="str">
-        <v>20%</v>
-      </c>
-      <c r="C6" t="str">
-        <v>No policy management, claims, or agent commission tracking</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Hospital (large / multi-specialty)</v>
-      </c>
-      <c r="B7" t="str">
-        <v>40%</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Current healthcare is clinic-level — missing OT scheduling, LIMS, pharmacy</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-  </mergeCells>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>